<commit_message>
Se genera cambio para aplicar los diferentes archivos por cada solicitud
</commit_message>
<xml_diff>
--- a/backend/src/assets/templates/SOLICITUDES.xlsx
+++ b/backend/src/assets/templates/SOLICITUDES.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\camig\MIENTRAS TANTO\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3e335d3f3ef462b1/Documentos/COSAS U/SEMESTRE 9/PRACTICAS/PROYECTO/BACKEND/PRACTICAS-BACK/backend/src/assets/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2A38DDB7-65CE-4AAA-8329-2C1FF3710B5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="8_{2A38DDB7-65CE-4AAA-8329-2C1FF3710B5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{56CBC75C-8A31-4786-80A3-3FA1486B078E}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{F2F517B1-4DB8-440A-BC86-F71603E3430E}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>N</t>
   </si>
@@ -61,13 +61,28 @@
   </si>
   <si>
     <t>DETALLE NOVEDAD</t>
+  </si>
+  <si>
+    <t>JORNADA EMPLEADO</t>
+  </si>
+  <si>
+    <t>CONCEPTO</t>
+  </si>
+  <si>
+    <t>CON_CODIGO</t>
+  </si>
+  <si>
+    <t>UNIDADES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FECHA NOVEDAD </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -82,8 +97,15 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -94,6 +116,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF002060"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF002060"/>
+        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
@@ -124,10 +152,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -518,7 +552,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CF83409-D84A-4693-A9F0-9171F3784A8E}">
-  <dimension ref="A5:H5"/>
+  <dimension ref="A5:M5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.140625" customWidth="1"/>
@@ -528,7 +562,7 @@
     <col min="8" max="8" width="28.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="1:8" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" ht="22.5" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
@@ -552,6 +586,21 @@
       </c>
       <c r="H5" s="1" t="s">
         <v>7</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="M5" s="3" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Se genera mejora en logica para descargue correcto de plantillas
</commit_message>
<xml_diff>
--- a/backend/src/assets/templates/SOLICITUDES.xlsx
+++ b/backend/src/assets/templates/SOLICITUDES.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3e335d3f3ef462b1/Documentos/COSAS U/SEMESTRE 9/PRACTICAS/PROYECTO/BACKEND/PRACTICAS-BACK/backend/src/assets/templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\camig\OneDrive\Documentos\COSAS U\SEMESTRE 9\PRACTICAS\PROYECTO\BACKEND\PRACTICAS-BACK\backend\src\assets\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="8_{2A38DDB7-65CE-4AAA-8329-2C1FF3710B5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{56CBC75C-8A31-4786-80A3-3FA1486B078E}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C371745A-CC61-4023-98BD-6BB116D00442}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{F2F517B1-4DB8-440A-BC86-F71603E3430E}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>N</t>
   </si>
@@ -61,21 +61,6 @@
   </si>
   <si>
     <t>DETALLE NOVEDAD</t>
-  </si>
-  <si>
-    <t>JORNADA EMPLEADO</t>
-  </si>
-  <si>
-    <t>CONCEPTO</t>
-  </si>
-  <si>
-    <t>CON_CODIGO</t>
-  </si>
-  <si>
-    <t>UNIDADES</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FECHA NOVEDAD </t>
   </si>
 </sst>
 </file>
@@ -120,7 +105,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF002060"/>
+        <fgColor theme="0"/>
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
@@ -157,10 +142,10 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -587,21 +572,11 @@
       <c r="H5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I5" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="K5" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="L5" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="M5" s="3" t="s">
-        <v>12</v>
-      </c>
+      <c r="I5" s="2"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+      <c r="L5" s="3"/>
+      <c r="M5" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>